<commit_message>
Added new dis8 code + adjusted dis3 +  retuned cen
</commit_message>
<xml_diff>
--- a/TDS_simulation_code/ANDES_Dutch_2035_mpc_cen.xlsx
+++ b/TDS_simulation_code/ANDES_Dutch_2035_mpc_cen.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piete\Documents\pieter\school\studie\Master\THESIS\CODE\MPC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piete\Documents\pieter\school\studie\Master\THESIS\CODE\MPC_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2002FC36-5E3A-4883-8D8A-124FFE4A23A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0C0A181-0E87-431E-A613-CC3AE8D1B379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28020" yWindow="780" windowWidth="21600" windowHeight="11295" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bus" sheetId="1" r:id="rId1"/>
@@ -7837,7 +7837,7 @@
         <v>90</v>
       </c>
       <c r="AK2">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="AL2">
         <v>1</v>
@@ -7925,7 +7925,7 @@
         <v>90</v>
       </c>
       <c r="AK3">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="AL3">
         <v>1</v>
@@ -8013,7 +8013,7 @@
         <v>90</v>
       </c>
       <c r="AK4">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="AL4">
         <v>1</v>
@@ -8101,7 +8101,7 @@
         <v>90</v>
       </c>
       <c r="AK5">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="AL5">
         <v>1</v>
@@ -8189,7 +8189,7 @@
         <v>90</v>
       </c>
       <c r="AK6">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="AL6">
         <v>1</v>
@@ -8277,7 +8277,7 @@
         <v>90</v>
       </c>
       <c r="AK7">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="AL7">
         <v>1</v>
@@ -8365,7 +8365,7 @@
         <v>90</v>
       </c>
       <c r="AK8">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="AL8">
         <v>1</v>
@@ -8453,7 +8453,7 @@
         <v>90</v>
       </c>
       <c r="AK9">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="AL9">
         <v>1</v>

</xml_diff>